<commit_message>
Add role-based attribute interpolation model
</commit_message>
<xml_diff>
--- a/support/docs/reference/scenario_6_=LOVE_member_roles.xlsx
+++ b/support/docs/reference/scenario_6_=LOVE_member_roles.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06C48708-4297-4455-9CBB-8BAE557E392A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D5602912-EB6E-4AD4-A64B-90B488063C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6220" yWindow="1130" windowWidth="30090" windowHeight="16820" xr2:uid="{34BF7C6B-7A81-444F-A303-C5D172F385AE}"/>
+    <workbookView xWindow="6220" yWindow="1130" windowWidth="30090" windowHeight="16820" xr2:uid="{843A4F0B-8986-419E-AC63-54A673379148}"/>
   </bookViews>
   <sheets>
     <sheet name="Roles" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
     <t>content</t>
   </si>
   <si>
-    <t>sns</t>
+    <t>streaming</t>
   </si>
   <si>
     <t>style</t>
@@ -326,7 +326,7 @@
                   <a14:compatExt spid="_x0000_s1025"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E7005640-8FA5-17AE-7A6B-1854F2801ACB}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2690242B-F2A0-5D00-43F7-EAC1C051525E}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -403,7 +403,7 @@
                   <a14:compatExt spid="_x0000_s1026"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DD65789-E6CD-0AE7-C278-9E39F8102976}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5FAA267-2AAA-6F66-8C2E-8E0DB92625BB}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -480,7 +480,7 @@
                   <a14:compatExt spid="_x0000_s1027"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC9AEADB-908B-5CCA-A479-F994A1305160}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54767856-8D73-29CA-7C5A-6FFFB88B9F4B}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -557,7 +557,7 @@
                   <a14:compatExt spid="_x0000_s1028"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A26B394B-20CE-06CA-D6B4-C7720A802D5A}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{627B4729-CD7D-D167-2BEE-85EC221CBDD5}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -634,7 +634,7 @@
                   <a14:compatExt spid="_x0000_s1029"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{011AD6E6-5B83-BF79-CC71-C590AE327BAF}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAD35E0E-F504-F43F-A499-31EBC672D360}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -711,7 +711,7 @@
                   <a14:compatExt spid="_x0000_s1030"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B208F37-AEC8-83F5-7D69-5F6D4E71D4D0}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88533990-7287-1473-25C7-467E36A96F0B}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -788,7 +788,7 @@
                   <a14:compatExt spid="_x0000_s1031"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{578531B1-118C-BB15-07AB-73E1BFC40FC5}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09362F61-9EFB-311A-98C6-B8A02559339A}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -865,7 +865,7 @@
                   <a14:compatExt spid="_x0000_s1032"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96552C4A-CD35-916C-2EBA-310C01889233}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67C1F098-54C1-F3B9-E562-2CE44751F1DF}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -942,7 +942,7 @@
                   <a14:compatExt spid="_x0000_s1033"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08AF1D31-9971-BD07-9305-D6AB5DE99D09}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B30C686-DBC7-70CC-36E6-1EF21900CDB4}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1019,7 +1019,7 @@
                   <a14:compatExt spid="_x0000_s1034"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{537EE03C-F6D1-79B9-B2B5-B2C3712AE977}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18E24D7F-FA9A-AB08-4ADF-C4CB603E9A73}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1372,7 +1372,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9840FB11-B14E-487B-B52B-CC6EBF4EB85D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF29FF18-B5F2-4DCB-8FE2-F59F379A69DA}">
   <dimension ref="A1:T11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1390,7 +1390,7 @@
     <col min="12" max="12" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="4.54296875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="4.7265625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="63.36328125" bestFit="1" customWidth="1"/>
@@ -1476,15 +1476,6 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="O2">
-        <v>5</v>
-      </c>
-      <c r="P2">
-        <v>5</v>
-      </c>
       <c r="R2" t="s">
         <v>22</v>
       </c>
@@ -1512,14 +1503,8 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="O3">
-        <v>5</v>
-      </c>
-      <c r="P3">
-        <v>5</v>
-      </c>
       <c r="Q3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R3" t="s">
         <v>26</v>
@@ -1548,12 +1533,6 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
-      <c r="O4">
-        <v>5</v>
-      </c>
-      <c r="P4">
-        <v>5</v>
-      </c>
       <c r="R4" t="s">
         <v>30</v>
       </c>
@@ -1590,12 +1569,6 @@
       <c r="M5">
         <v>2</v>
       </c>
-      <c r="O5">
-        <v>4</v>
-      </c>
-      <c r="P5">
-        <v>3</v>
-      </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
@@ -1629,12 +1602,6 @@
       <c r="M6">
         <v>3</v>
       </c>
-      <c r="O6">
-        <v>5</v>
-      </c>
-      <c r="P6">
-        <v>5</v>
-      </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -1668,12 +1635,6 @@
       <c r="M7">
         <v>3</v>
       </c>
-      <c r="O7">
-        <v>5</v>
-      </c>
-      <c r="P7">
-        <v>5</v>
-      </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
@@ -1698,12 +1659,6 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
-      <c r="O8">
-        <v>5</v>
-      </c>
-      <c r="P8">
-        <v>5</v>
-      </c>
       <c r="Q8">
         <v>2</v>
       </c>
@@ -1743,12 +1698,6 @@
       <c r="M9">
         <v>3</v>
       </c>
-      <c r="O9">
-        <v>5</v>
-      </c>
-      <c r="P9">
-        <v>5</v>
-      </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -1776,12 +1725,6 @@
       <c r="K10">
         <v>4</v>
       </c>
-      <c r="O10">
-        <v>5</v>
-      </c>
-      <c r="P10">
-        <v>5</v>
-      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
@@ -1815,21 +1758,15 @@
       <c r="M11">
         <v>5</v>
       </c>
-      <c r="O11">
-        <v>2</v>
-      </c>
-      <c r="P11">
-        <v>5</v>
-      </c>
       <c r="R11" t="s">
         <v>53</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T11" xr:uid="{9840FB11-B14E-487B-B52B-CC6EBF4EB85D}"/>
+  <autoFilter ref="A1:T11" xr:uid="{CF29FF18-B5F2-4DCB-8FE2-F59F379A69DA}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Weight" error="Role weights must be blank or one of 1, 2, 3, 4, 5." promptTitle="Role Weight" prompt="Select 1-5, or leave blank if the role does not apply." sqref="I2:Q11" xr:uid="{AD9A768D-4F12-476A-9199-7C9748085393}">
-      <formula1>"1,2,3,4,5"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Weight" error="Role weights must be blank or one of 0, 1, 2, 3, 4, 5." promptTitle="Role Weight" prompt="Select 0-5, or leave blank if the role does not apply. 0 is treated as no role." sqref="I2:Q11" xr:uid="{44F0B5C6-F75A-4529-A8B7-618546B26D1B}">
+      <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>